<commit_message>
Risk Register V0.7: score RSK-021 P2 x I3 (owner decision, consistent with RSK-009 and RSK-016)
</commit_message>
<xml_diff>
--- a/docs/risk/Risk Register/Risk Register V0.7.xlsx
+++ b/docs/risk/Risk Register/Risk Register V0.7.xlsx
@@ -3099,8 +3099,12 @@
           <t>Repeated auth.login.failure events in auditLog for one account or one source within minutes; CON-019 adversarial testing targeting login; any successful login following a run of failures.</t>
         </is>
       </c>
-      <c r="F23" s="78" t="n"/>
-      <c r="G23" s="78" t="n"/>
+      <c r="F23" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="78" t="n">
+        <v>3</v>
+      </c>
       <c r="H23" s="79">
         <f>IF(OR(F23="",G23=""),"",F23*G23)</f>
         <v/>
@@ -3136,7 +3140,7 @@
       </c>
       <c r="O23" s="64" t="inlineStr">
         <is>
-          <t>New at M3 — raised by DEC-018 (11/10/2026). Not yet scored: probability and impact to be set by the owner consistently with the other access-control risks (RSK-009 is scored P2 × I3).</t>
+          <t>New at M3 — raised by DEC-018 (11/10/2026). Scored P2 × I3 = 6 (High) by the owner, consistent with RSK-009 and RSK-016, the same class of risk. P2: the risk rests on an unconfirmed assumption, that the slow hash caps the guess rate, which has not been measured. Not P3: CON-019 adversarial testing is planned, not an indicator already present.</t>
         </is>
       </c>
     </row>

</xml_diff>